<commit_message>
se añadio las SLA
</commit_message>
<xml_diff>
--- a/Selva Viva/Rasgos_SelvaViva_unificado.xlsx
+++ b/Selva Viva/Rasgos_SelvaViva_unificado.xlsx
@@ -15,6 +15,9 @@
     <sheet name="Rasgos_SelvaViva_unificado" sheetId="1" r:id="rId1"/>
     <sheet name="Filas_a_revisar" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Rasgos_SelvaViva_unificado!$A$1:$BB$63</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -1003,6 +1006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:BB63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1178,7 +1182,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -1300,7 +1304,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -1422,7 +1426,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>54</v>
       </c>
@@ -1541,7 +1545,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>54</v>
       </c>
@@ -1663,7 +1667,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -1782,7 +1786,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -1901,7 +1905,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -2023,7 +2027,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -2142,7 +2146,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -2264,7 +2268,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -2386,7 +2390,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -2502,7 +2506,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -2624,7 +2628,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -2743,7 +2747,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>54</v>
       </c>
@@ -2862,7 +2866,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>54</v>
       </c>
@@ -3094,7 +3098,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>54</v>
       </c>
@@ -3213,7 +3217,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -3335,7 +3339,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="20" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -3454,7 +3458,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="21" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>54</v>
       </c>
@@ -3552,7 +3556,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>54</v>
       </c>
@@ -3654,7 +3658,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -3773,7 +3777,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="24" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -3892,7 +3896,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="25" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>54</v>
       </c>
@@ -4011,7 +4015,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="26" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>54</v>
       </c>
@@ -4103,7 +4107,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="27" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>54</v>
       </c>
@@ -4225,7 +4229,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="28" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>54</v>
       </c>
@@ -4344,7 +4348,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="29" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>54</v>
       </c>
@@ -4469,7 +4473,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>54</v>
       </c>
@@ -4588,7 +4592,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="31" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>54</v>
       </c>
@@ -4713,7 +4717,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="32" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>54</v>
       </c>
@@ -4835,7 +4839,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="33" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>54</v>
       </c>
@@ -5052,7 +5056,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="35" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>54</v>
       </c>
@@ -5171,7 +5175,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="36" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>54</v>
       </c>
@@ -5266,7 +5270,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="37" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>54</v>
       </c>
@@ -5385,7 +5389,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>54</v>
       </c>
@@ -5507,7 +5511,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="39" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>54</v>
       </c>
@@ -5626,7 +5630,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="40" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>54</v>
       </c>
@@ -5730,7 +5734,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="41" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>54</v>
       </c>
@@ -5852,7 +5856,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="42" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>54</v>
       </c>
@@ -5974,7 +5978,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="43" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>54</v>
       </c>
@@ -6096,7 +6100,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>54</v>
       </c>
@@ -6218,7 +6222,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>54</v>
       </c>
@@ -6343,7 +6347,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="46" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -6465,7 +6469,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="47" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>54</v>
       </c>
@@ -6587,7 +6591,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="48" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -6783,7 +6787,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>54</v>
       </c>
@@ -6820,6 +6824,9 @@
       <c r="N50">
         <v>10.220000000000001</v>
       </c>
+      <c r="O50">
+        <v>1096.538</v>
+      </c>
       <c r="R50">
         <v>393.22816467872258</v>
       </c>
@@ -6893,7 +6900,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="51" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>54</v>
       </c>
@@ -6930,6 +6937,9 @@
       <c r="N51">
         <v>10.050000000000001</v>
       </c>
+      <c r="O51">
+        <v>883.26800000000003</v>
+      </c>
       <c r="R51">
         <v>406.06060606060612</v>
       </c>
@@ -7003,7 +7013,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="52" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>54</v>
       </c>
@@ -7040,6 +7050,9 @@
       <c r="N52">
         <v>12.91</v>
       </c>
+      <c r="O52">
+        <v>1270.2429999999999</v>
+      </c>
       <c r="R52">
         <v>443.18571918983872</v>
       </c>
@@ -7116,7 +7129,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="53" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>54</v>
       </c>
@@ -7153,6 +7166,9 @@
       <c r="N53">
         <v>5.84</v>
       </c>
+      <c r="O53">
+        <v>1005.977</v>
+      </c>
       <c r="R53">
         <v>290.98156452416538</v>
       </c>
@@ -7226,7 +7242,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="54" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>54</v>
       </c>
@@ -7263,6 +7279,9 @@
       <c r="N54">
         <v>12.73</v>
       </c>
+      <c r="O54">
+        <v>1442.249</v>
+      </c>
       <c r="R54">
         <v>451.25841900035448</v>
       </c>
@@ -7336,7 +7355,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="55" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>54</v>
       </c>
@@ -7373,6 +7392,9 @@
       <c r="N55">
         <v>8.2200000000000006</v>
       </c>
+      <c r="O55">
+        <v>782.18200000000002</v>
+      </c>
       <c r="R55">
         <v>404.12979351032448</v>
       </c>
@@ -7455,7 +7477,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="56" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>54</v>
       </c>
@@ -7492,6 +7514,9 @@
       <c r="N56">
         <v>10.75</v>
       </c>
+      <c r="O56">
+        <v>1212.402</v>
+      </c>
       <c r="R56">
         <v>446.61404237640221</v>
       </c>
@@ -7571,7 +7596,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="57" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>54</v>
       </c>
@@ -7605,6 +7630,9 @@
       <c r="N57">
         <v>10.75</v>
       </c>
+      <c r="O57">
+        <v>1379.91</v>
+      </c>
       <c r="R57">
         <v>437.88187372708762</v>
       </c>
@@ -7690,7 +7718,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="58" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>54</v>
       </c>
@@ -7727,6 +7755,9 @@
       <c r="N58">
         <v>11.83</v>
       </c>
+      <c r="O58">
+        <v>1920.3679999999999</v>
+      </c>
       <c r="R58">
         <v>334.65346534653457</v>
       </c>
@@ -7812,7 +7843,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="59" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>54</v>
       </c>
@@ -7849,6 +7880,9 @@
       <c r="N59">
         <v>16.03</v>
       </c>
+      <c r="O59">
+        <v>1633.528</v>
+      </c>
       <c r="R59">
         <v>460.36760482481338</v>
       </c>
@@ -7934,7 +7968,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="60" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>54</v>
       </c>
@@ -7971,6 +8005,9 @@
       <c r="N60">
         <v>12.57</v>
       </c>
+      <c r="O60">
+        <v>858.76300000000003</v>
+      </c>
       <c r="R60">
         <v>553.74449339207047</v>
       </c>
@@ -8050,7 +8087,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="61" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>54</v>
       </c>
@@ -8087,6 +8124,9 @@
       <c r="N61">
         <v>14.62</v>
       </c>
+      <c r="O61">
+        <v>1521.2829999999999</v>
+      </c>
       <c r="R61">
         <v>497.61742682096673</v>
       </c>
@@ -8166,7 +8206,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="62" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>54</v>
       </c>
@@ -8203,6 +8243,9 @@
       <c r="N62">
         <v>13.92</v>
       </c>
+      <c r="O62">
+        <v>1725.4110000000001</v>
+      </c>
       <c r="R62">
         <v>329.15582880113499</v>
       </c>
@@ -8282,7 +8325,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="63" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:54" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>54</v>
       </c>
@@ -8316,6 +8359,9 @@
       <c r="N63">
         <v>19.8</v>
       </c>
+      <c r="O63">
+        <v>1616.3009999999999</v>
+      </c>
       <c r="R63">
         <v>374.64522232734151</v>
       </c>
@@ -8405,6 +8451,11 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BB63">
+    <filterColumn colId="14">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>